<commit_message>
implemented customers and customers behavior and injected raw data on them an its working perfectly
</commit_message>
<xml_diff>
--- a/generator/output/master/suppliers.xlsx
+++ b/generator/output/master/suppliers.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Laikipia</t>
+          <t>LAIKIPIA</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1003,11 +1003,7 @@
           <t>Grace Njoroge</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>+254715881177</t>
-        </is>
-      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>support@ungagroup.ac.ke</t>
@@ -1183,7 +1179,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Laikipia</t>
+          <t>laikipia</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -3360,11 +3356,7 @@
           <t>+254714501641</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>admin@cadburykenya.co.ke</t>
-        </is>
-      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>Laikipia</t>
@@ -3479,7 +3471,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Bungoma</t>
+          <t>bungoma</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -3510,7 +3502,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Colgate Palmolive</t>
+          <t xml:space="preserve"> Colgate Palmolive</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -3678,7 +3670,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Johnson &amp; Johnson Kenya</t>
+          <t xml:space="preserve"> Johnson &amp; Johnson Kenya</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3691,11 +3683,7 @@
           <t>Grace Odhiambo</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>+254740120324</t>
-        </is>
-      </c>
+      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>admin@johnsonjohnsonkenya.ac.ke</t>
@@ -4645,7 +4633,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>+254793536390</t>
+          <t>+254718265409</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -4928,11 +4916,7 @@
           <t>+254758885339</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>support@smartheartkenya.ke</t>
-        </is>
-      </c>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>Machakos</t>
@@ -6045,7 +6029,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>+254768916118</t>
+          <t>+254748760021</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -6559,7 +6543,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Kilifi</t>
+          <t>kilifi</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">

</xml_diff>